<commit_message>
Separating by event not tag
</commit_message>
<xml_diff>
--- a/tagsheet_to_tidbits2025/data/Sander's PIT CODES.xlsx
+++ b/tagsheet_to_tidbits2025/data/Sander's PIT CODES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umainesystem-my.sharepoint.com/personal/sander_elliott_maine_edu/Documents/Desktop/Github/Sturgeon_TidBits/tagsheet_to_tidbits2025/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{87E30D02-C812-421C-A0AA-2F4032EB8D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D613798-27E4-42F6-8F60-023531AB6DF7}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{87E30D02-C812-421C-A0AA-2F4032EB8D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAA3E067-F1CF-4C23-BA8A-A0A1D0F9DE7B}"/>
   <bookViews>
-    <workbookView xWindow="29070" yWindow="0" windowWidth="28530" windowHeight="15480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28755" yWindow="285" windowWidth="28530" windowHeight="15480" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trip" sheetId="7" r:id="rId1"/>
@@ -1148,7 +1148,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
@@ -1176,7 +1176,6 @@
     <xf numFmtId="0" fontId="17" fillId="13" borderId="11" xfId="22" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1339,6 +1338,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3356,7 +3359,7 @@
         <f>VALUE(RIGHT(E2,6))</f>
         <v>201133</v>
       </c>
-      <c r="H2" s="15">
+      <c r="H2">
         <v>1645258</v>
       </c>
       <c r="I2" t="s">
@@ -3380,7 +3383,7 @@
         <f t="shared" ref="F3:F51" si="0">VALUE(RIGHT(E3,6))</f>
         <v>201127</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3">
         <v>1645259</v>
       </c>
       <c r="I3" t="s">
@@ -3413,7 +3416,7 @@
         <f t="shared" si="0"/>
         <v>201134</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4">
         <v>1645260</v>
       </c>
       <c r="I4" t="s">
@@ -3449,7 +3452,7 @@
         <f t="shared" si="0"/>
         <v>201128</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5">
         <v>1645261</v>
       </c>
       <c r="I5" t="s">
@@ -3485,7 +3488,7 @@
         <f t="shared" si="0"/>
         <v>201129</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6">
         <v>1645262</v>
       </c>
       <c r="I6" t="s">
@@ -3521,7 +3524,7 @@
         <f t="shared" si="0"/>
         <v>201131</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7">
         <v>1645263</v>
       </c>
       <c r="I7" t="s">
@@ -3557,7 +3560,7 @@
         <f t="shared" si="0"/>
         <v>201130</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8">
         <v>1645264</v>
       </c>
       <c r="I8" t="s">
@@ -3593,7 +3596,7 @@
         <f t="shared" si="0"/>
         <v>201132</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9">
         <v>1645265</v>
       </c>
       <c r="I9" t="s">
@@ -3629,7 +3632,7 @@
         <f t="shared" si="0"/>
         <v>201212</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10">
         <v>1645266</v>
       </c>
       <c r="I10" t="s">
@@ -3665,7 +3668,7 @@
         <f t="shared" si="0"/>
         <v>201215</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11">
         <v>1645267</v>
       </c>
       <c r="I11" t="s">
@@ -3701,7 +3704,7 @@
         <f t="shared" si="0"/>
         <v>201213</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12">
         <v>1645268</v>
       </c>
       <c r="I12" t="s">
@@ -3737,7 +3740,7 @@
         <f t="shared" si="0"/>
         <v>201214</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13">
         <v>1645269</v>
       </c>
       <c r="I13" t="s">
@@ -3773,7 +3776,7 @@
         <f t="shared" si="0"/>
         <v>201216</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14">
         <v>1645270</v>
       </c>
       <c r="I14" t="s">
@@ -3809,7 +3812,7 @@
         <f t="shared" si="0"/>
         <v>201217</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15">
         <v>1645271</v>
       </c>
       <c r="I15" t="s">
@@ -3845,7 +3848,7 @@
         <f t="shared" si="0"/>
         <v>201218</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16">
         <v>1645272</v>
       </c>
       <c r="I16" t="s">
@@ -3881,7 +3884,7 @@
         <f t="shared" si="0"/>
         <v>201219</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17">
         <v>1645273</v>
       </c>
       <c r="I17" t="s">
@@ -3917,7 +3920,7 @@
         <f t="shared" si="0"/>
         <v>201220</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18">
         <v>1645274</v>
       </c>
       <c r="I18" t="s">
@@ -3953,7 +3956,7 @@
         <f t="shared" si="0"/>
         <v>201223</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19">
         <v>1645275</v>
       </c>
       <c r="I19" t="s">
@@ -3989,7 +3992,7 @@
         <f t="shared" si="0"/>
         <v>201222</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20">
         <v>1645276</v>
       </c>
       <c r="I20" t="s">
@@ -4025,7 +4028,7 @@
         <f t="shared" si="0"/>
         <v>201221</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21">
         <v>1645277</v>
       </c>
       <c r="I21" t="s">
@@ -4061,7 +4064,7 @@
         <f t="shared" si="0"/>
         <v>201224</v>
       </c>
-      <c r="H22" s="15">
+      <c r="H22">
         <v>1645278</v>
       </c>
       <c r="I22" t="s">
@@ -4097,7 +4100,7 @@
         <f t="shared" si="0"/>
         <v>201225</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H23">
         <v>1645279</v>
       </c>
       <c r="I23" t="s">
@@ -4133,7 +4136,7 @@
         <f t="shared" si="0"/>
         <v>201226</v>
       </c>
-      <c r="H24" s="15">
+      <c r="H24">
         <v>1645280</v>
       </c>
       <c r="I24" t="s">
@@ -4169,7 +4172,7 @@
         <f t="shared" si="0"/>
         <v>201227</v>
       </c>
-      <c r="H25" s="15">
+      <c r="H25">
         <v>1645281</v>
       </c>
       <c r="I25" t="s">
@@ -4205,7 +4208,7 @@
         <f t="shared" si="0"/>
         <v>201228</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26">
         <v>1645282</v>
       </c>
       <c r="I26" t="s">
@@ -4241,7 +4244,7 @@
         <f t="shared" si="0"/>
         <v>201229</v>
       </c>
-      <c r="H27" s="15">
+      <c r="H27">
         <v>1645283</v>
       </c>
       <c r="I27" t="s">
@@ -4277,7 +4280,7 @@
         <f t="shared" si="0"/>
         <v>201232</v>
       </c>
-      <c r="H28" s="15">
+      <c r="H28">
         <v>1645284</v>
       </c>
       <c r="I28" t="s">
@@ -4313,7 +4316,7 @@
         <f t="shared" si="0"/>
         <v>201231</v>
       </c>
-      <c r="H29" s="15">
+      <c r="H29">
         <v>1645285</v>
       </c>
       <c r="I29" t="s">
@@ -4349,7 +4352,7 @@
         <f t="shared" si="0"/>
         <v>201230</v>
       </c>
-      <c r="H30" s="15">
+      <c r="H30">
         <v>1645286</v>
       </c>
       <c r="I30" t="s">
@@ -4385,7 +4388,7 @@
         <f t="shared" si="0"/>
         <v>201235</v>
       </c>
-      <c r="H31" s="15">
+      <c r="H31">
         <v>1645287</v>
       </c>
       <c r="I31" t="s">
@@ -4421,7 +4424,7 @@
         <f t="shared" si="0"/>
         <v>201234</v>
       </c>
-      <c r="H32" s="15">
+      <c r="H32">
         <v>1645288</v>
       </c>
       <c r="I32" t="s">
@@ -4457,7 +4460,7 @@
         <f t="shared" si="0"/>
         <v>201233</v>
       </c>
-      <c r="H33" s="15">
+      <c r="H33">
         <v>1645289</v>
       </c>
       <c r="I33" t="s">
@@ -4493,7 +4496,7 @@
         <f t="shared" si="0"/>
         <v>201238</v>
       </c>
-      <c r="H34" s="15">
+      <c r="H34">
         <v>1645290</v>
       </c>
       <c r="I34" t="s">
@@ -4529,7 +4532,7 @@
         <f t="shared" si="0"/>
         <v>201237</v>
       </c>
-      <c r="H35" s="15">
+      <c r="H35">
         <v>1645291</v>
       </c>
       <c r="I35" t="s">
@@ -4565,7 +4568,7 @@
         <f t="shared" si="0"/>
         <v>201236</v>
       </c>
-      <c r="H36" s="15">
+      <c r="H36">
         <v>1645292</v>
       </c>
       <c r="I36" t="s">
@@ -4601,7 +4604,7 @@
         <f t="shared" si="0"/>
         <v>201239</v>
       </c>
-      <c r="H37" s="15">
+      <c r="H37">
         <v>1645293</v>
       </c>
       <c r="I37" t="s">
@@ -4637,7 +4640,7 @@
         <f t="shared" si="0"/>
         <v>201240</v>
       </c>
-      <c r="H38" s="15">
+      <c r="H38">
         <v>1645294</v>
       </c>
       <c r="I38" t="s">
@@ -4673,7 +4676,7 @@
         <f t="shared" si="0"/>
         <v>201241</v>
       </c>
-      <c r="H39" s="15">
+      <c r="H39">
         <v>1645295</v>
       </c>
       <c r="I39" t="s">
@@ -4709,7 +4712,7 @@
         <f t="shared" si="0"/>
         <v>201244</v>
       </c>
-      <c r="H40" s="15">
+      <c r="H40">
         <v>1645296</v>
       </c>
       <c r="I40" t="s">
@@ -4745,7 +4748,7 @@
         <f t="shared" si="0"/>
         <v>201243</v>
       </c>
-      <c r="H41" s="15">
+      <c r="H41">
         <v>1645297</v>
       </c>
       <c r="I41" t="s">
@@ -4781,7 +4784,7 @@
         <f t="shared" si="0"/>
         <v>201242</v>
       </c>
-      <c r="H42" s="15">
+      <c r="H42">
         <v>1645298</v>
       </c>
       <c r="I42" t="s">
@@ -4817,7 +4820,7 @@
         <f t="shared" si="0"/>
         <v>201247</v>
       </c>
-      <c r="H43" s="15">
+      <c r="H43">
         <v>1645299</v>
       </c>
       <c r="I43" t="s">
@@ -5141,7 +5144,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+      <c r="A2">
         <v>1645258</v>
       </c>
       <c r="B2" t="s">
@@ -5149,7 +5152,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
+      <c r="A3">
         <v>1645259</v>
       </c>
       <c r="B3" t="s">
@@ -5157,7 +5160,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4">
         <v>1645260</v>
       </c>
       <c r="B4" t="s">
@@ -5165,7 +5168,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+      <c r="A5">
         <v>1645261</v>
       </c>
       <c r="B5" t="s">
@@ -5173,7 +5176,7 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="A6">
         <v>1645262</v>
       </c>
       <c r="B6" t="s">
@@ -5181,7 +5184,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+      <c r="A7">
         <v>1645263</v>
       </c>
       <c r="B7" t="s">
@@ -5189,7 +5192,7 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8">
         <v>1645264</v>
       </c>
       <c r="B8" t="s">
@@ -5197,7 +5200,7 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9">
         <v>1645265</v>
       </c>
       <c r="B9" t="s">
@@ -5205,7 +5208,7 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10">
         <v>1645266</v>
       </c>
       <c r="B10" t="s">
@@ -5213,7 +5216,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11">
         <v>1645267</v>
       </c>
       <c r="B11" t="s">
@@ -5221,7 +5224,7 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12">
         <v>1645268</v>
       </c>
       <c r="B12" t="s">
@@ -5229,7 +5232,7 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13">
         <v>1645269</v>
       </c>
       <c r="B13" t="s">
@@ -5237,7 +5240,7 @@
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14">
         <v>1645270</v>
       </c>
       <c r="B14" t="s">
@@ -5245,7 +5248,7 @@
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15">
         <v>1645271</v>
       </c>
       <c r="B15" t="s">
@@ -5253,7 +5256,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16">
         <v>1645272</v>
       </c>
       <c r="B16" t="s">
@@ -5261,7 +5264,7 @@
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17">
         <v>1645273</v>
       </c>
       <c r="B17" t="s">
@@ -5269,7 +5272,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18">
         <v>1645274</v>
       </c>
       <c r="B18" t="s">
@@ -5277,7 +5280,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19">
         <v>1645275</v>
       </c>
       <c r="B19" t="s">
@@ -5285,7 +5288,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20">
         <v>1645276</v>
       </c>
       <c r="B20" t="s">
@@ -5293,7 +5296,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21">
         <v>1645277</v>
       </c>
       <c r="B21" t="s">
@@ -5301,7 +5304,7 @@
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22">
         <v>1645278</v>
       </c>
       <c r="B22" t="s">
@@ -5309,7 +5312,7 @@
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23">
         <v>1645279</v>
       </c>
       <c r="B23" t="s">
@@ -5317,7 +5320,7 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24">
         <v>1645280</v>
       </c>
       <c r="B24" t="s">
@@ -5325,7 +5328,7 @@
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25">
         <v>1645281</v>
       </c>
       <c r="B25" t="s">
@@ -5333,7 +5336,7 @@
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
+      <c r="A26">
         <v>1645282</v>
       </c>
       <c r="B26" t="s">
@@ -5341,7 +5344,7 @@
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27">
         <v>1645283</v>
       </c>
       <c r="B27" t="s">
@@ -5349,7 +5352,7 @@
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
+      <c r="A28">
         <v>1645284</v>
       </c>
       <c r="B28" t="s">
@@ -5357,7 +5360,7 @@
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29">
         <v>1645285</v>
       </c>
       <c r="B29" t="s">
@@ -5365,7 +5368,7 @@
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
+      <c r="A30">
         <v>1645286</v>
       </c>
       <c r="B30" t="s">
@@ -5373,7 +5376,7 @@
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31">
         <v>1645287</v>
       </c>
       <c r="B31" t="s">
@@ -5381,7 +5384,7 @@
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
+      <c r="A32">
         <v>1645288</v>
       </c>
       <c r="B32" t="s">
@@ -5389,7 +5392,7 @@
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33">
         <v>1645289</v>
       </c>
       <c r="B33" t="s">
@@ -5397,7 +5400,7 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34">
         <v>1645290</v>
       </c>
       <c r="B34" t="s">
@@ -5405,7 +5408,7 @@
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35">
         <v>1645291</v>
       </c>
       <c r="B35" t="s">
@@ -5413,7 +5416,7 @@
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
+      <c r="A36">
         <v>1645292</v>
       </c>
       <c r="B36" t="s">
@@ -5421,7 +5424,7 @@
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
+      <c r="A37">
         <v>1645293</v>
       </c>
       <c r="B37" t="s">
@@ -5429,7 +5432,7 @@
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
+      <c r="A38">
         <v>1645294</v>
       </c>
       <c r="B38" t="s">
@@ -5437,7 +5440,7 @@
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="15">
+      <c r="A39">
         <v>1645295</v>
       </c>
       <c r="B39" t="s">
@@ -5445,7 +5448,7 @@
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="15">
+      <c r="A40">
         <v>1645296</v>
       </c>
       <c r="B40" t="s">
@@ -5453,7 +5456,7 @@
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="15">
+      <c r="A41">
         <v>1645297</v>
       </c>
       <c r="B41" t="s">
@@ -5461,7 +5464,7 @@
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="15">
+      <c r="A42">
         <v>1645298</v>
       </c>
       <c r="B42" t="s">
@@ -5469,7 +5472,7 @@
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="15">
+      <c r="A43">
         <v>1645299</v>
       </c>
       <c r="B43" t="s">
@@ -9187,7 +9190,7 @@
         <v>140</v>
       </c>
       <c r="C12">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12">
         <v>201251</v>
@@ -9215,7 +9218,7 @@
       </c>
       <c r="N12" t="str">
         <f>IF(C12="", "", _xlfn.XLOOKUP(C12, Sheet1!A:A, Sheet1!B:B, ""))</f>
-        <v>3DD.003E185F84</v>
+        <v>3DD.003E185F67</v>
       </c>
       <c r="O12" t="str">
         <f>IF(D12="", "", _xlfn.XLOOKUP(D12, Sheet1!F:F, Sheet1!E:E, ""))</f>
@@ -9607,7 +9610,6 @@
       <c r="F38" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="Q2:Q100">
     <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;$B2, $Q2&lt;&gt;"UKN", $Q2&lt;&gt;"", $B2&lt;&gt;"")</formula>

</xml_diff>